<commit_message>
fix: bind cooperative decisions to observed sessions and retire radio work
Reject stale votes and duplicate transitions with persisted private resynchronization.
Preserve concurrent session-lifetime and host-election corrections.
Guard radio negotiations, final shutdown and controller push-to-talk across interruptions.
Add domain, HTTP adapter and client regressions with dated source and workbook evidence.
</commit_message>
<xml_diff>
--- a/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
+++ b/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R7aa352db576a4051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="2" r:id="Rd9635000d0304bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Rae797f56ab404c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="2" r:id="R0ed974cbb7b64e80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctifs 29-10" sheetId="3" r:id="R3258857577bc4cd8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="11">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0"/>
+  </x:numFmts>
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -74,8 +79,53 @@
       <x:color rgb="FF68778C"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF14243B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:color rgb="FF14243B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF50627B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF82520E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF14243B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF50627B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FF28415F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF50627B"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,15 +147,45 @@
         <x:fgColor rgb="FF28415F"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF28415F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF28415F"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5DDE5"/>
+      </x:left>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -203,11 +283,118 @@
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="14">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCE8F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDF3E8"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF0CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF0E5F3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:fill>
         <x:patternFill patternType="solid">
@@ -236,6 +423,62 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9A2525"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFDE8E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF82520E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF82520E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF82520E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF82520E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF1D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF66778D"/>
+      </x:font>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -251,6 +494,22 @@
     <x:tableColumn id="6" name="Critère de validation"/>
     <x:tableColumn id="7" name="Preuve / limite"/>
     <x:tableColumn id="8" name="Source"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Correctifs20261029" displayName="Correctifs20261029" ref="A8:H16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Correction"/>
+    <x:tableColumn id="3" name="Statut"/>
+    <x:tableColumn id="4" name="Critère de validation"/>
+    <x:tableColumn id="5" name="Preuve"/>
+    <x:tableColumn id="6" name="Limite"/>
+    <x:tableColumn id="7" name="Suite"/>
+    <x:tableColumn id="8" name="Sources du lot"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1404,16 +1663,16 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D28">
-    <x:cfRule type="expression" dxfId="0" priority="1">
+    <x:cfRule type="expression" dxfId="4" priority="1">
       <x:formula>$D5="Existant — CI passée"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1" priority="2">
+    <x:cfRule type="expression" dxfId="5" priority="2">
       <x:formula>$D5="Réalisé — tests locaux"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="2" priority="3">
+    <x:cfRule type="expression" dxfId="6" priority="3">
       <x:formula>$D5="À valider"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="3" priority="4">
+    <x:cfRule type="expression" dxfId="7" priority="4">
       <x:formula>$D5="À réaliser"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -1427,7 +1686,912 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad69b7af39224d90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135c63bd58fc476f"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF28415F"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="49" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="52"/>
+      <x:c r="B1" s="52"/>
+      <x:c r="C1" s="52"/>
+      <x:c r="D1" s="52"/>
+      <x:c r="E1" s="52"/>
+      <x:c r="F1" s="52"/>
+      <x:c r="G1" s="52"/>
+      <x:c r="H1" s="52"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="54" t="str">
+        <x:v>PARALLAXE — CORRECTIFS DU 29 OCTOBRE 2026</x:v>
+      </x:c>
+      <x:c r="B2" s="54"/>
+      <x:c r="C2" s="54"/>
+      <x:c r="D2" s="54"/>
+      <x:c r="E2" s="54"/>
+      <x:c r="F2" s="54"/>
+      <x:c r="G2" s="54"/>
+      <x:c r="H2" s="54"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="52" t="str">
+        <x:v>Origine du lot</x:v>
+      </x:c>
+      <x:c r="B3" s="52" t="str">
+        <x:v>1a7196f0151b3e755edc5670d8d571a9ec9e065c</x:v>
+      </x:c>
+      <x:c r="C3" s="52"/>
+      <x:c r="D3" s="52" t="str">
+        <x:v>Base intégrée</x:v>
+      </x:c>
+      <x:c r="E3" s="52" t="str">
+        <x:v>f738ab9a54df2b6b651c179c5e9b035ca626719c</x:v>
+      </x:c>
+      <x:c r="F3" s="52"/>
+      <x:c r="G3" s="52"/>
+      <x:c r="H3" s="52"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="52" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B4" s="55" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C4" s="52"/>
+      <x:c r="D4" s="52" t="str">
+        <x:v>PR 2</x:v>
+      </x:c>
+      <x:c r="E4" s="52" t="str">
+        <x:v>https://github.com/darknigthmare/Parallaxe_Protocole9/pull/2</x:v>
+      </x:c>
+      <x:c r="F4" s="52"/>
+      <x:c r="G4" s="52"/>
+      <x:c r="H4" s="52"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="56" t="str">
+        <x:v>Les onglets précédents restent les instantanés du 28 octobre. Les identifiants ci-dessous appartiennent au lot du 29 octobre.</x:v>
+      </x:c>
+      <x:c r="B5" s="56"/>
+      <x:c r="C5" s="56"/>
+      <x:c r="D5" s="56"/>
+      <x:c r="E5" s="56"/>
+      <x:c r="F5" s="56"/>
+      <x:c r="G5" s="56"/>
+      <x:c r="H5" s="56"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="58" t="str">
+        <x:v>Sources GitHub : 0.2.1, trois lieux. Texte publié du Site : 0.4.0, quatre lieux. Sources du Site non récupérées.</x:v>
+      </x:c>
+      <x:c r="B6" s="58"/>
+      <x:c r="C6" s="58"/>
+      <x:c r="D6" s="58"/>
+      <x:c r="E6" s="58"/>
+      <x:c r="F6" s="58"/>
+      <x:c r="G6" s="58"/>
+      <x:c r="H6" s="58"/>
+    </x:row>
+    <x:row r="7" ht="10" customHeight="1">
+      <x:c r="A7" s="52"/>
+      <x:c r="B7" s="52"/>
+      <x:c r="C7" s="52"/>
+      <x:c r="D7" s="52"/>
+      <x:c r="E7" s="52"/>
+      <x:c r="F7" s="52"/>
+      <x:c r="G7" s="52"/>
+      <x:c r="H7" s="52"/>
+    </x:row>
+    <x:row r="8" ht="31" customHeight="1">
+      <x:c r="A8" s="62" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B8" s="62" t="str">
+        <x:v>Correction</x:v>
+      </x:c>
+      <x:c r="C8" s="62" t="str">
+        <x:v>Statut</x:v>
+      </x:c>
+      <x:c r="D8" s="62" t="str">
+        <x:v>Critère de validation</x:v>
+      </x:c>
+      <x:c r="E8" s="62" t="str">
+        <x:v>Preuve</x:v>
+      </x:c>
+      <x:c r="F8" s="62" t="str">
+        <x:v>Limite</x:v>
+      </x:c>
+      <x:c r="G8" s="62" t="str">
+        <x:v>Suite</x:v>
+      </x:c>
+      <x:c r="H8" s="62" t="str">
+        <x:v>Sources du lot</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="103" customHeight="1">
+      <x:c r="A9" s="64" t="str">
+        <x:v>COOP05</x:v>
+      </x:c>
+      <x:c r="B9" s="64" t="str">
+        <x:v>Rejeter les votes retardés</x:v>
+      </x:c>
+      <x:c r="C9" s="63" t="str">
+        <x:v>Réalisé, tests locaux réussis</x:v>
+      </x:c>
+      <x:c r="D9" s="63" t="str">
+        <x:v>Un vote capturé dans un ancien decisionEpoch ne vote pas dans le passage suivant. Un vote dans le contexte courant reste possible.</x:v>
+      </x:c>
+      <x:c r="E9" s="63" t="str">
+        <x:v>Domaine intégré : 66/66 tests réussis, dont 16 tests d'actions. Adaptateurs : 5/5. Rejet HTTP 409 des décisions périmées avec état courant privé.</x:v>
+      </x:c>
+      <x:c r="F9" s="63" t="str">
+        <x:v>Résultat local sur les règles partagées. La CI du commit livré et une partie humaine restent à contrôler.</x:v>
+      </x:c>
+      <x:c r="G9" s="63" t="str">
+        <x:v>Vérifier la resynchronisation de l'interface avec plusieurs navigateurs et le frontend compilé.</x:v>
+      </x:c>
+      <x:c r="H9" s="65" t="str">
+        <x:v>src/game/session.ts
+tests/session-actions.test.mjs
+tests/session-adapters.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="103" customHeight="1">
+      <x:c r="A10" s="64" t="str">
+        <x:v>COOP06</x:v>
+      </x:c>
+      <x:c r="B10" s="64" t="str">
+        <x:v>Conserver la référence du nouveau lieu</x:v>
+      </x:c>
+      <x:c r="C10" s="63" t="str">
+        <x:v>Réalisé, tests locaux réussis</x:v>
+      </x:c>
+      <x:c r="D10" s="63" t="str">
+        <x:v>Un second next reçu après le changement de secteur ne saute pas la phase de référence du nouveau lieu.</x:v>
+      </x:c>
+      <x:c r="E10" s="63" t="str">
+        <x:v>Régression du double next dans les 16 tests d'actions. Les 5 tests d'adaptateurs couvrent aussi la concurrence CAS et trois phases de référence via HTTP.</x:v>
+      </x:c>
+      <x:c r="F10" s="63" t="str">
+        <x:v>Le test protège la transition logique. Il ne prouve pas le rendu ou la lisibilité du nouveau lieu.</x:v>
+      </x:c>
+      <x:c r="G10" s="63" t="str">
+        <x:v>Vérifier le parcours complet et l'affichage de la référence sur les clients.</x:v>
+      </x:c>
+      <x:c r="H10" s="65" t="str">
+        <x:v>src/game/session.ts
+tests/session-actions.test.mjs
+tests/session-adapters.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="103" customHeight="1">
+      <x:c r="A11" s="64" t="str">
+        <x:v>COOP07</x:v>
+      </x:c>
+      <x:c r="B11" s="64" t="str">
+        <x:v>Invalider la décision après une absence</x:v>
+      </x:c>
+      <x:c r="C11" s="63" t="str">
+        <x:v>Réalisé, tests locaux réussis</x:v>
+      </x:c>
+      <x:c r="D11" s="63" t="str">
+        <x:v>Une interruption de présence invalide l'ancien contexte, même sans vote enregistré. Le retour exige une décision fraîche.</x:v>
+      </x:c>
+      <x:c r="E11" s="63" t="str">
+        <x:v>Domaine intégré : 66/66. Régressions d'absence sans vote et d'invalidation unique. Les adaptateurs vérifient la persistance du nettoyage avant le rejet 409.</x:v>
+      </x:c>
+      <x:c r="F11" s="63" t="str">
+        <x:v>Les pauses réseau réelles et la reprise d'une partie humaine ne sont pas validées par ces tests.</x:v>
+      </x:c>
+      <x:c r="G11" s="63" t="str">
+        <x:v>Tester une absence, une reconnexion et un vote retardé sur plusieurs clients.</x:v>
+      </x:c>
+      <x:c r="H11" s="65" t="str">
+        <x:v>src/game/session.ts
+tests/session-actions.test.mjs
+tests/session-resilience.test.mjs
+tests/session-adapters.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="103" customHeight="1">
+      <x:c r="A12" s="64" t="str">
+        <x:v>RAD07</x:v>
+      </x:c>
+      <x:c r="B12" s="64" t="str">
+        <x:v>Annuler les négociations radio périmées</x:v>
+      </x:c>
+      <x:c r="C12" s="63" t="str">
+        <x:v>Réalisé, tests locaux réussis</x:v>
+      </x:c>
+      <x:c r="D12" s="63" t="str">
+        <x:v>Ignorer les suites et rejets RTC périmés après extinction, dispose, reconnexion, départ du pair ou changement de son radioEpoch. Un pair courant continue à négocier.</x:v>
+      </x:c>
+      <x:c r="E12" s="63" t="str">
+        <x:v>Radio : 29/29. Quatre régressions supplémentaires ont échoué avant correction puis réussi après : rejets tardifs RTC d'un pair parti ou remplacé.</x:v>
+      </x:c>
+      <x:c r="F12" s="63" t="str">
+        <x:v>API audio et WebRTC simulées. Aucun microphone réel ni relais TURN entre réseaux n'est validé.</x:v>
+      </x:c>
+      <x:c r="G12" s="63" t="str">
+        <x:v>Vérifier extinction et reconnexion avec de vrais appareils et un relais TURN entre réseaux.</x:v>
+      </x:c>
+      <x:c r="H12" s="65" t="str">
+        <x:v>src/game/radio.ts
+tests/radio.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="103" customHeight="1">
+      <x:c r="A13" s="64" t="str">
+        <x:v>INPUT01</x:v>
+      </x:c>
+      <x:c r="B13" s="64" t="str">
+        <x:v>Sécuriser le push-to-talk manette</x:v>
+      </x:c>
+      <x:c r="C13" s="63" t="str">
+        <x:v>Réalisé, tests locaux réussis</x:v>
+      </x:c>
+      <x:c r="D13" s="63" t="str">
+        <x:v>blur, onglet masqué ou pause coupe le PTT, même entre deux images. Le retour exige de relâcher le bouton puis de réappuyer.</x:v>
+      </x:c>
+      <x:c r="E13" s="63" t="str">
+        <x:v>PTT : 11/11, dont 7 tests d'automate et 4 tests des vrais callbacks exécutés par harnais. Les tests client couvrent aussi pause, changement de session et perte réseau entre deux images.</x:v>
+      </x:c>
+      <x:c r="F13" s="63" t="str">
+        <x:v>API navigateur simulées par harnais. Aucune manette physique ni aucun microphone réel testé.</x:v>
+      </x:c>
+      <x:c r="G13" s="63" t="str">
+        <x:v>Rejouer perte de focus, pause et changement d'onglet avec manette et microphone physiques.</x:v>
+      </x:c>
+      <x:c r="H13" s="65" t="str">
+        <x:v>app/game.tsx
+src/game/radio-input.ts
+tests/radio-input.test.mjs
+tests/session-scope.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="103" customHeight="1">
+      <x:c r="A14" s="64" t="str">
+        <x:v>CLIENT01</x:v>
+      </x:c>
+      <x:c r="B14" s="64" t="str">
+        <x:v>Compléter le cycle de vie des sessions client</x:v>
+      </x:c>
+      <x:c r="C14" s="63" t="str">
+        <x:v>Protection préservée et complétée</x:v>
+      </x:c>
+      <x:c r="D14" s="63" t="str">
+        <x:v>Une fermeture ou annulation create/join retire la requête. Les anciens callbacks radio ne changent pas la session reprise. L'arrêt final utilise les anciens identifiants sans réadopter sa réponse.</x:v>
+      </x:c>
+      <x:c r="E14" s="63" t="str">
+        <x:v>SessionScope : 60/60, dont 34 tests concurrents conservés et 26 complémentaires. Annulations, reprise de la même identité, callbacks radio et paquet final d'arrêt couverts.</x:v>
+      </x:c>
+      <x:c r="F14" s="63" t="str">
+        <x:v>Callbacks du code exécutés dans un harnais avec API navigateur simulées. Le rendu React dans un navigateur réel n'est pas validé.</x:v>
+      </x:c>
+      <x:c r="G14" s="63" t="str">
+        <x:v>Jouer les transitions coopération, annulation, solo et reprise dans plusieurs navigateurs.</x:v>
+      </x:c>
+      <x:c r="H14" s="65" t="str">
+        <x:v>app/game.tsx
+src/game/session-scope.ts
+tests/session-scope.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="103" customHeight="1">
+      <x:c r="A15" s="64" t="str">
+        <x:v>CLIENT02</x:v>
+      </x:c>
+      <x:c r="B15" s="64" t="str">
+        <x:v>Lier chaque action à son contexte affiché</x:v>
+      </x:c>
+      <x:c r="C15" s="63" t="str">
+        <x:v>Réalisé, tests locaux réussis</x:v>
+      </x:c>
+      <x:c r="D15" s="63" t="str">
+        <x:v>Une action issue d'un ancien affichage ou d'une ancienne visite ne part pas avec les identifiants du salon courant, même si decisionEpoch est identique.</x:v>
+      </x:c>
+      <x:c r="E15" s="63" t="str">
+        <x:v>Inclus dans les 60 tests SessionScope : contexte de rendu, visite, identité, rejet 409 sans réessai automatique et protection d'une nouvelle fenêtre après réponse tardive.</x:v>
+      </x:c>
+      <x:c r="F15" s="63" t="str">
+        <x:v>Harnais client et HTTP contrôlés. Aucune partie humaine sur plusieurs appareils n'est attestée par ces tests.</x:v>
+      </x:c>
+      <x:c r="G15" s="63" t="str">
+        <x:v>Vérifier vote, passage suivant et reprise du même salon avec une interface compilée et plusieurs clients.</x:v>
+      </x:c>
+      <x:c r="H15" s="65" t="str">
+        <x:v>app/game.tsx
+src/game/session-scope.ts
+tests/session-scope.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="103" customHeight="1">
+      <x:c r="A16" s="64" t="str">
+        <x:v>SRC01</x:v>
+      </x:c>
+      <x:c r="B16" s="64" t="str">
+        <x:v>Récupérer les sources du Site</x:v>
+      </x:c>
+      <x:c r="C16" s="63" t="str">
+        <x:v>Bloqué par accès réseau</x:v>
+      </x:c>
+      <x:c r="D16" s="63" t="str">
+        <x:v>Récupérer le sourceSHA de la version 7, comparer avec GitHub 0.2.1 et vérifier le lien avec le texte publié 0.4.0.</x:v>
+      </x:c>
+      <x:c r="E16" s="63" t="str">
+        <x:v>Version 7 et sourceSHA connus. Texte publié du 28 octobre : 0.4.0 et quatre lieux, dont Chalet de service. GitHub : 0.2.1 et trois lieux.</x:v>
+      </x:c>
+      <x:c r="F16" s="63" t="str">
+        <x:v>git.chatgpt-team.site inaccessible. Connexion browser-proxy indisponible. La comparaison du code n'est pas réalisée.</x:v>
+      </x:c>
+      <x:c r="G16" s="63" t="str">
+        <x:v>Rétablir l'accès au dépôt source ou obtenir son archive, puis comparer avant toute livraison remplaçant le Site.</x:v>
+      </x:c>
+      <x:c r="H16" s="65" t="str">
+        <x:v>docs/SOURCE_RECONCILIATION_2026-10-29.md
+Métadonnées du Site, version 7
+Texte de publication capturé le 28 octobre 2026
+package.json
+src/game/levels.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="52"/>
+      <x:c r="B17" s="52"/>
+      <x:c r="C17" s="52"/>
+      <x:c r="D17" s="52"/>
+      <x:c r="E17" s="52"/>
+      <x:c r="F17" s="52"/>
+      <x:c r="G17" s="52"/>
+      <x:c r="H17" s="52"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="52"/>
+      <x:c r="B18" s="52"/>
+      <x:c r="C18" s="52"/>
+      <x:c r="D18" s="52"/>
+      <x:c r="E18" s="52"/>
+      <x:c r="F18" s="52"/>
+      <x:c r="G18" s="52"/>
+      <x:c r="H18" s="52"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="66" t="str">
+        <x:v>VALIDATIONS DU LOT</x:v>
+      </x:c>
+      <x:c r="B19" s="66"/>
+      <x:c r="C19" s="66"/>
+      <x:c r="D19" s="66"/>
+      <x:c r="E19" s="66"/>
+      <x:c r="F19" s="66"/>
+      <x:c r="G19" s="66"/>
+      <x:c r="H19" s="66"/>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="62" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B20" s="62" t="str">
+        <x:v>Contrôle</x:v>
+      </x:c>
+      <x:c r="C20" s="62" t="str">
+        <x:v>Statut</x:v>
+      </x:c>
+      <x:c r="D20" s="62" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="E20" s="62" t="str">
+        <x:v>Prévus / total</x:v>
+      </x:c>
+      <x:c r="F20" s="62" t="str">
+        <x:v>Commande</x:v>
+      </x:c>
+      <x:c r="G20" s="62" t="str">
+        <x:v>Résultat observé</x:v>
+      </x:c>
+      <x:c r="H20" s="62" t="str">
+        <x:v>Limite de validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="65" customHeight="1">
+      <x:c r="A21" s="63" t="str">
+        <x:v>DOMAIN</x:v>
+      </x:c>
+      <x:c r="B21" s="63" t="str">
+        <x:v>Domaine partagé</x:v>
+      </x:c>
+      <x:c r="C21" s="63" t="str">
+        <x:v>Réussi localement</x:v>
+      </x:c>
+      <x:c r="D21" s="68" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E21" s="68" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F21" s="71" t="str">
+        <x:v>npm test, sous-ensemble domaine</x:v>
+      </x:c>
+      <x:c r="G21" s="63" t="str">
+        <x:v>Règles : 17. Résilience : 33, dont 5 tests concurrents conservés. Actions : 16.</x:v>
+      </x:c>
+      <x:c r="H21" s="63" t="str">
+        <x:v>Règles partagées, sans validation graphique ou matérielle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="65" customHeight="1">
+      <x:c r="A22" s="69" t="str">
+        <x:v>PTT</x:v>
+      </x:c>
+      <x:c r="B22" s="69" t="str">
+        <x:v>Entrées PTT manette</x:v>
+      </x:c>
+      <x:c r="C22" s="69" t="str">
+        <x:v>Réussi localement</x:v>
+      </x:c>
+      <x:c r="D22" s="70" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E22" s="70" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F22" s="72" t="str">
+        <x:v>node tests/radio-input.test.mjs</x:v>
+      </x:c>
+      <x:c r="G22" s="69" t="str">
+        <x:v>7 tests d'automate et 4 tests des vrais callbacks exécutés par harnais. L'interruption entre deux images ne réarme pas un bouton maintenu.</x:v>
+      </x:c>
+      <x:c r="H22" s="69" t="str">
+        <x:v>API navigateur simulées. Aucune manette physique ni aucun microphone réel testé.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="65" customHeight="1">
+      <x:c r="A23" s="63" t="str">
+        <x:v>RADIO</x:v>
+      </x:c>
+      <x:c r="B23" s="63" t="str">
+        <x:v>Cycle de vie radio</x:v>
+      </x:c>
+      <x:c r="C23" s="63" t="str">
+        <x:v>Réussi localement</x:v>
+      </x:c>
+      <x:c r="D23" s="68" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E23" s="68" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F23" s="71" t="str">
+        <x:v>npm run test:radio</x:v>
+      </x:c>
+      <x:c r="G23" s="63" t="str">
+        <x:v>25 tests précédents et 4 régressions de rejets RTC tardifs après départ ou remplacement du pair. Ces 4 défauts étaient reproduits avant correction.</x:v>
+      </x:c>
+      <x:c r="H23" s="63" t="str">
+        <x:v>API audio et WebRTC simulées. Aucun microphone réel validé.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="65" customHeight="1">
+      <x:c r="A24" s="69" t="str">
+        <x:v>HTTP</x:v>
+      </x:c>
+      <x:c r="B24" s="69" t="str">
+        <x:v>Adaptateurs D1 et HTTP Node</x:v>
+      </x:c>
+      <x:c r="C24" s="69" t="str">
+        <x:v>Réussi localement</x:v>
+      </x:c>
+      <x:c r="D24" s="70" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E24" s="70" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F24" s="72" t="str">
+        <x:v>node tests/session-adapters.test.mjs</x:v>
+      </x:c>
+      <x:c r="G24" s="69" t="str">
+        <x:v>4 tests des vrais handlers D1 sur stockage CAS simulé. 1 scénario vrai HTTP Node sur localhost : 4 clients, 9 consensus, 3 références, rejets 409.</x:v>
+      </x:c>
+      <x:c r="H24" s="69" t="str">
+        <x:v>Sources exécutées sans annotations de types et page HTML de test. Frontend compilé et D1 déployé non validés.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="65" customHeight="1">
+      <x:c r="A25" s="63" t="str">
+        <x:v>CLIENT</x:v>
+      </x:c>
+      <x:c r="B25" s="63" t="str">
+        <x:v>Sessions client SessionScope</x:v>
+      </x:c>
+      <x:c r="C25" s="63" t="str">
+        <x:v>Réussi localement</x:v>
+      </x:c>
+      <x:c r="D25" s="68" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E25" s="68" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F25" s="71" t="str">
+        <x:v>npm run test:session-client</x:v>
+      </x:c>
+      <x:c r="G25" s="63" t="str">
+        <x:v>34 tests concurrents conservés et 26 complémentaires. Avec 66 tests de domaine et 5 adaptateurs, npm test totalise 131/131.</x:v>
+      </x:c>
+      <x:c r="H25" s="63" t="str">
+        <x:v>Vrais callbacks du code dans un harnais avec API navigateur simulées. Aucun contrôle du rendu React en navigateur.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="65" customHeight="1">
+      <x:c r="A26" s="69" t="str">
+        <x:v>BUILD</x:v>
+      </x:c>
+      <x:c r="B26" s="69" t="str">
+        <x:v>Typage et compilation</x:v>
+      </x:c>
+      <x:c r="C26" s="69" t="str">
+        <x:v>En attente CI</x:v>
+      </x:c>
+      <x:c r="D26" s="70"/>
+      <x:c r="E26" s="70"/>
+      <x:c r="F26" s="72" t="str">
+        <x:v>npm run typecheck ; npm run build:local ; npm run test:portable</x:v>
+      </x:c>
+      <x:c r="G26" s="69" t="str">
+        <x:v>Typage, compilation et contrôle du portable compilé restent à valider en CI.</x:v>
+      </x:c>
+      <x:c r="H26" s="69" t="str">
+        <x:v>Le test HTTP depuis les sources ne remplace pas la compilation du frontend.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="65" customHeight="1">
+      <x:c r="A27" s="63" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="B27" s="63" t="str">
+        <x:v>CI du commit livré</x:v>
+      </x:c>
+      <x:c r="C27" s="63" t="str">
+        <x:v>En attente CI</x:v>
+      </x:c>
+      <x:c r="D27" s="68"/>
+      <x:c r="E27" s="68"/>
+      <x:c r="F27" s="71" t="str">
+        <x:v>GitHub Actions sur la PR 2</x:v>
+      </x:c>
+      <x:c r="G27" s="63" t="str">
+        <x:v>En attente sur le commit publié. La CI doit aussi vérifier 4 tests d'actions radio, 59 de configuration et 11 de scène.</x:v>
+      </x:c>
+      <x:c r="H27" s="63" t="str">
+        <x:v>Aucun résultat de CI attribué avant exécution sur le commit exact. La scène CPU ne valide pas le GPU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="65" customHeight="1">
+      <x:c r="A28" s="69" t="str">
+        <x:v>GPU</x:v>
+      </x:c>
+      <x:c r="B28" s="69" t="str">
+        <x:v>GPU et reflets</x:v>
+      </x:c>
+      <x:c r="C28" s="69" t="str">
+        <x:v>Non exécuté</x:v>
+      </x:c>
+      <x:c r="D28" s="70"/>
+      <x:c r="E28" s="70"/>
+      <x:c r="F28" s="72" t="str">
+        <x:v>Essai matériel</x:v>
+      </x:c>
+      <x:c r="G28" s="69" t="str">
+        <x:v>Aucun contrôle GPU revendiqué dans cette passe.</x:v>
+      </x:c>
+      <x:c r="H28" s="69" t="str">
+        <x:v>Corps, reflets, anomalies et performances restent à vérifier visuellement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="65" customHeight="1">
+      <x:c r="A29" s="63" t="str">
+        <x:v>MIC</x:v>
+      </x:c>
+      <x:c r="B29" s="63" t="str">
+        <x:v>Microphones réels</x:v>
+      </x:c>
+      <x:c r="C29" s="63" t="str">
+        <x:v>Non exécuté</x:v>
+      </x:c>
+      <x:c r="D29" s="68"/>
+      <x:c r="E29" s="68"/>
+      <x:c r="F29" s="71" t="str">
+        <x:v>Essai matériel</x:v>
+      </x:c>
+      <x:c r="G29" s="63" t="str">
+        <x:v>Aucun essai de voix réelle revendiqué.</x:v>
+      </x:c>
+      <x:c r="H29" s="63" t="str">
+        <x:v>Intelligibilité, permission, coupure et reprise à tester sur appareils.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="65" customHeight="1">
+      <x:c r="A30" s="69" t="str">
+        <x:v>TURN</x:v>
+      </x:c>
+      <x:c r="B30" s="69" t="str">
+        <x:v>TURN entre réseaux</x:v>
+      </x:c>
+      <x:c r="C30" s="69" t="str">
+        <x:v>Non exécuté</x:v>
+      </x:c>
+      <x:c r="D30" s="70"/>
+      <x:c r="E30" s="70"/>
+      <x:c r="F30" s="72" t="str">
+        <x:v>Essai matériel</x:v>
+      </x:c>
+      <x:c r="G30" s="69" t="str">
+        <x:v>Aucune connexion relayée entre réseaux vérifiée.</x:v>
+      </x:c>
+      <x:c r="H30" s="69" t="str">
+        <x:v>Tester avec un relais configuré et deux réseaux distincts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="52"/>
+      <x:c r="B31" s="52"/>
+      <x:c r="C31" s="52"/>
+      <x:c r="D31" s="52"/>
+      <x:c r="E31" s="52"/>
+      <x:c r="F31" s="52"/>
+      <x:c r="G31" s="52"/>
+      <x:c r="H31" s="52"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="52"/>
+      <x:c r="B32" s="52"/>
+      <x:c r="C32" s="52"/>
+      <x:c r="D32" s="52"/>
+      <x:c r="E32" s="52"/>
+      <x:c r="F32" s="52"/>
+      <x:c r="G32" s="52"/>
+      <x:c r="H32" s="52"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="66" t="str">
+        <x:v>ÉCART DE SOURCES À RÉCONCILIER</x:v>
+      </x:c>
+      <x:c r="B33" s="66"/>
+      <x:c r="C33" s="66"/>
+      <x:c r="D33" s="66"/>
+      <x:c r="E33" s="66"/>
+      <x:c r="F33" s="66"/>
+      <x:c r="G33" s="66"/>
+      <x:c r="H33" s="66"/>
+    </x:row>
+    <x:row r="34" ht="30" customHeight="1">
+      <x:c r="A34" s="62" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B34" s="62" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="C34" s="62" t="str">
+        <x:v>Lieux annoncés</x:v>
+      </x:c>
+      <x:c r="D34" s="62" t="str">
+        <x:v>Version sauvegardée</x:v>
+      </x:c>
+      <x:c r="E34" s="62" t="str">
+        <x:v>Preuve disponible</x:v>
+      </x:c>
+      <x:c r="F34" s="62" t="str">
+        <x:v>Limite</x:v>
+      </x:c>
+      <x:c r="G34" s="62" t="str">
+        <x:v>Suite</x:v>
+      </x:c>
+      <x:c r="H34" s="62" t="str">
+        <x:v>Référence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="81" customHeight="1">
+      <x:c r="A35" s="63" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="B35" s="63" t="str">
+        <x:v>0.2.1</x:v>
+      </x:c>
+      <x:c r="C35" s="68" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D35" s="68"/>
+      <x:c r="E35" s="71" t="str">
+        <x:v>Code du dépôt examiné à partir de la base indiquée.</x:v>
+      </x:c>
+      <x:c r="F35" s="63" t="str">
+        <x:v>La version GitHub ne prouve pas le contenu du Site 0.4.0.</x:v>
+      </x:c>
+      <x:c r="G35" s="63" t="str">
+        <x:v>Conserver la base des correctifs isolés.</x:v>
+      </x:c>
+      <x:c r="H35" s="63" t="str">
+        <x:v>package.json
+src/game/levels.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="81" customHeight="1">
+      <x:c r="A36" s="73" t="str">
+        <x:v>Site</x:v>
+      </x:c>
+      <x:c r="B36" s="73" t="str">
+        <x:v>0.4.0</x:v>
+      </x:c>
+      <x:c r="C36" s="74" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D36" s="74" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E36" s="75" t="str">
+        <x:v>Métadonnées et texte capturé le 28 octobre. Chalet de service affiché.</x:v>
+      </x:c>
+      <x:c r="F36" s="73" t="str">
+        <x:v>Code non récupéré. La version sauvegardée 7 ne prouve pas la version actuellement déployée. Accès réseau bloqué.</x:v>
+      </x:c>
+      <x:c r="G36" s="73" t="str">
+        <x:v>Récupérer le code ou une archive, puis comparer avant remplacement du Site.</x:v>
+      </x:c>
+      <x:c r="H36" s="73" t="str">
+        <x:v>6c8784e0cf5d64f6386f3448434b0bc659d3fc15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="52"/>
+      <x:c r="B37" s="52"/>
+      <x:c r="C37" s="52"/>
+      <x:c r="D37" s="52"/>
+      <x:c r="E37" s="52"/>
+      <x:c r="F37" s="52"/>
+      <x:c r="G37" s="52"/>
+      <x:c r="H37" s="52"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="52"/>
+      <x:c r="B38" s="52"/>
+      <x:c r="C38" s="52"/>
+      <x:c r="D38" s="52"/>
+      <x:c r="E38" s="52"/>
+      <x:c r="F38" s="52"/>
+      <x:c r="G38" s="52"/>
+      <x:c r="H38" s="52"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="76" t="str">
+        <x:v>Livraison</x:v>
+      </x:c>
+      <x:c r="B39" s="77" t="str">
+        <x:v>Pas de fusion ni de déploiement dans cette passe.</x:v>
+      </x:c>
+      <x:c r="C39" s="77"/>
+      <x:c r="D39" s="77"/>
+      <x:c r="E39" s="77"/>
+      <x:c r="F39" s="77"/>
+      <x:c r="G39" s="77"/>
+      <x:c r="H39" s="77"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="76" t="str">
+        <x:v>Classeur source</x:v>
+      </x:c>
+      <x:c r="B40" s="77" t="str">
+        <x:v>docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx</x:v>
+      </x:c>
+      <x:c r="C40" s="77"/>
+      <x:c r="D40" s="77"/>
+      <x:c r="E40" s="77"/>
+      <x:c r="F40" s="77"/>
+      <x:c r="G40" s="77"/>
+      <x:c r="H40" s="77"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="76" t="str">
+        <x:v>Empreinte Git</x:v>
+      </x:c>
+      <x:c r="B41" s="77" t="str">
+        <x:v>27846a00639f0611e2ee4b4eaff2e653769a0e16</x:v>
+      </x:c>
+      <x:c r="C41" s="77"/>
+      <x:c r="D41" s="77"/>
+      <x:c r="E41" s="77"/>
+      <x:c r="F41" s="77"/>
+      <x:c r="G41" s="77"/>
+      <x:c r="H41" s="77"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="76" t="str">
+        <x:v>Suivi détaillé</x:v>
+      </x:c>
+      <x:c r="B42" s="77" t="str">
+        <x:v>docs/suivi-correctifs-20261029.json</x:v>
+      </x:c>
+      <x:c r="C42" s="77"/>
+      <x:c r="D42" s="77"/>
+      <x:c r="E42" s="77"/>
+      <x:c r="F42" s="77"/>
+      <x:c r="G42" s="77"/>
+      <x:c r="H42" s="77"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="76" t="str">
+        <x:v>Preuve manquante</x:v>
+      </x:c>
+      <x:c r="B43" s="77" t="str">
+        <x:v>Les cellules numériques vides correspondent à un résultat non disponible ou à un essai non exécuté, pas à zéro réussite.</x:v>
+      </x:c>
+      <x:c r="C43" s="77"/>
+      <x:c r="D43" s="77"/>
+      <x:c r="E43" s="77"/>
+      <x:c r="F43" s="77"/>
+      <x:c r="G43" s="77"/>
+      <x:c r="H43" s="77"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="76" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="B44" s="77" t="str">
+        <x:v>docs/SOURCE_RECONCILIATION_2026-10-29.md</x:v>
+      </x:c>
+      <x:c r="C44" s="77"/>
+      <x:c r="D44" s="77"/>
+      <x:c r="E44" s="77"/>
+      <x:c r="F44" s="77"/>
+      <x:c r="G44" s="77"/>
+      <x:c r="H44" s="77"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="76" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="B45" s="77" t="str">
+        <x:v>docs/QA.md</x:v>
+      </x:c>
+      <x:c r="C45" s="77"/>
+      <x:c r="D45" s="77"/>
+      <x:c r="E45" s="77"/>
+      <x:c r="F45" s="77"/>
+      <x:c r="G45" s="77"/>
+      <x:c r="H45" s="77"/>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="C9:C16">
+    <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Bloqué"/>
+    <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="en cours"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C21:C30">
+    <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="En cours"/>
+    <x:cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="En attente"/>
+    <x:cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Non validé"/>
+    <x:cfRule type="containsText" dxfId="13" priority="6" operator="containsText" text="Non exécuté"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19bd297353c241ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record passing CI and preserve dated correction evidence
Tie QA and the tracking workbook to code f258c5b6 and workflow run 40884677504.
Record 234 passing Node tests, 11 CPU geometry checks and the compiled portable scenario.
Preserve workbook history and distinguish simulated validation from outstanding device tests.
</commit_message>
<xml_diff>
--- a/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
+++ b/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Rae797f56ab404c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="2" r:id="R0ed974cbb7b64e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctifs 29-10" sheetId="3" r:id="R3258857577bc4cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R0b19b9158c464378"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="2" r:id="Rf274adb891e642e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctifs 29-10" sheetId="3" r:id="R1daed0cc66c3480d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1686,7 +1686,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135c63bd58fc476f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R402255b052be4e12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1790,12 +1790,20 @@
       <x:c r="G6" s="58"/>
       <x:c r="H6" s="58"/>
     </x:row>
-    <x:row r="7" ht="10" customHeight="1">
-      <x:c r="A7" s="52"/>
-      <x:c r="B7" s="52"/>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="52" t="str">
+        <x:v>Code testé</x:v>
+      </x:c>
+      <x:c r="B7" s="52" t="str">
+        <x:v>f258c5b6bd99e24d6ef9650941fa6a86b162a1f0</x:v>
+      </x:c>
       <x:c r="C7" s="52"/>
-      <x:c r="D7" s="52"/>
-      <x:c r="E7" s="52"/>
+      <x:c r="D7" s="52" t="str">
+        <x:v>CI réussie sur ce code</x:v>
+      </x:c>
+      <x:c r="E7" s="52" t="str">
+        <x:v>https://github.com/darknigthmare/Parallaxe_Protocole9/actions/runs/40884677504</x:v>
+      </x:c>
       <x:c r="F7" s="52"/>
       <x:c r="G7" s="52"/>
       <x:c r="H7" s="52"/>
@@ -1834,7 +1842,7 @@
         <x:v>Rejeter les votes retardés</x:v>
       </x:c>
       <x:c r="C9" s="63" t="str">
-        <x:v>Réalisé, tests locaux réussis</x:v>
+        <x:v>Réalisé, confirmé en CI</x:v>
       </x:c>
       <x:c r="D9" s="63" t="str">
         <x:v>Un vote capturé dans un ancien decisionEpoch ne vote pas dans le passage suivant. Un vote dans le contexte courant reste possible.</x:v>
@@ -1843,7 +1851,7 @@
         <x:v>Domaine intégré : 66/66 tests réussis, dont 16 tests d'actions. Adaptateurs : 5/5. Rejet HTTP 409 des décisions périmées avec état courant privé.</x:v>
       </x:c>
       <x:c r="F9" s="63" t="str">
-        <x:v>Résultat local sur les règles partagées. La CI du commit livré et une partie humaine restent à contrôler.</x:v>
+        <x:v>Règles et HTTP vérifiés sur le commit testé. Stockage D1 simulé. La partie humaine sur plusieurs appareils reste à contrôler.</x:v>
       </x:c>
       <x:c r="G9" s="63" t="str">
         <x:v>Vérifier la resynchronisation de l'interface avec plusieurs navigateurs et le frontend compilé.</x:v>
@@ -1862,7 +1870,7 @@
         <x:v>Conserver la référence du nouveau lieu</x:v>
       </x:c>
       <x:c r="C10" s="63" t="str">
-        <x:v>Réalisé, tests locaux réussis</x:v>
+        <x:v>Réalisé, confirmé en CI</x:v>
       </x:c>
       <x:c r="D10" s="63" t="str">
         <x:v>Un second next reçu après le changement de secteur ne saute pas la phase de référence du nouveau lieu.</x:v>
@@ -1890,7 +1898,7 @@
         <x:v>Invalider la décision après une absence</x:v>
       </x:c>
       <x:c r="C11" s="63" t="str">
-        <x:v>Réalisé, tests locaux réussis</x:v>
+        <x:v>Réalisé, confirmé en CI</x:v>
       </x:c>
       <x:c r="D11" s="63" t="str">
         <x:v>Une interruption de présence invalide l'ancien contexte, même sans vote enregistré. Le retour exige une décision fraîche.</x:v>
@@ -1919,7 +1927,7 @@
         <x:v>Annuler les négociations radio périmées</x:v>
       </x:c>
       <x:c r="C12" s="63" t="str">
-        <x:v>Réalisé, tests locaux réussis</x:v>
+        <x:v>Réalisé, confirmé en CI</x:v>
       </x:c>
       <x:c r="D12" s="63" t="str">
         <x:v>Ignorer les suites et rejets RTC périmés après extinction, dispose, reconnexion, départ du pair ou changement de son radioEpoch. Un pair courant continue à négocier.</x:v>
@@ -1946,7 +1954,7 @@
         <x:v>Sécuriser le push-to-talk manette</x:v>
       </x:c>
       <x:c r="C13" s="63" t="str">
-        <x:v>Réalisé, tests locaux réussis</x:v>
+        <x:v>Réalisé, confirmé en CI</x:v>
       </x:c>
       <x:c r="D13" s="63" t="str">
         <x:v>blur, onglet masqué ou pause coupe le PTT, même entre deux images. Le retour exige de relâcher le bouton puis de réappuyer.</x:v>
@@ -1981,7 +1989,7 @@
         <x:v>Une fermeture ou annulation create/join retire la requête. Les anciens callbacks radio ne changent pas la session reprise. L'arrêt final utilise les anciens identifiants sans réadopter sa réponse.</x:v>
       </x:c>
       <x:c r="E14" s="63" t="str">
-        <x:v>SessionScope : 60/60, dont 34 tests concurrents conservés et 26 complémentaires. Annulations, reprise de la même identité, callbacks radio et paquet final d'arrêt couverts.</x:v>
+        <x:v>SessionScope : 60/60 en local puis en CI, dont 34 tests concurrents conservés et 26 complémentaires. Annulations, même identité, callbacks radio et arrêt final couverts.</x:v>
       </x:c>
       <x:c r="F14" s="63" t="str">
         <x:v>Callbacks du code exécutés dans un harnais avec API navigateur simulées. Le rendu React dans un navigateur réel n'est pas validé.</x:v>
@@ -2003,7 +2011,7 @@
         <x:v>Lier chaque action à son contexte affiché</x:v>
       </x:c>
       <x:c r="C15" s="63" t="str">
-        <x:v>Réalisé, tests locaux réussis</x:v>
+        <x:v>Réalisé, confirmé en CI</x:v>
       </x:c>
       <x:c r="D15" s="63" t="str">
         <x:v>Une action issue d'un ancien affichage ou d'une ancienne visite ne part pas avec les identifiants du salon courant, même si decisionEpoch est identique.</x:v>
@@ -2119,7 +2127,7 @@
         <x:v>Domaine partagé</x:v>
       </x:c>
       <x:c r="C21" s="63" t="str">
-        <x:v>Réussi localement</x:v>
+        <x:v>Réussi localement et en CI</x:v>
       </x:c>
       <x:c r="D21" s="68" t="n">
         <x:v>66</x:v>
@@ -2145,7 +2153,7 @@
         <x:v>Entrées PTT manette</x:v>
       </x:c>
       <x:c r="C22" s="69" t="str">
-        <x:v>Réussi localement</x:v>
+        <x:v>Réussi localement et en CI</x:v>
       </x:c>
       <x:c r="D22" s="70" t="n">
         <x:v>11</x:v>
@@ -2171,7 +2179,7 @@
         <x:v>Cycle de vie radio</x:v>
       </x:c>
       <x:c r="C23" s="63" t="str">
-        <x:v>Réussi localement</x:v>
+        <x:v>Réussi localement et en CI</x:v>
       </x:c>
       <x:c r="D23" s="68" t="n">
         <x:v>29</x:v>
@@ -2197,7 +2205,7 @@
         <x:v>Adaptateurs D1 et HTTP Node</x:v>
       </x:c>
       <x:c r="C24" s="69" t="str">
-        <x:v>Réussi localement</x:v>
+        <x:v>Réussi localement et en CI</x:v>
       </x:c>
       <x:c r="D24" s="70" t="n">
         <x:v>5</x:v>
@@ -2212,7 +2220,7 @@
         <x:v>4 tests des vrais handlers D1 sur stockage CAS simulé. 1 scénario vrai HTTP Node sur localhost : 4 clients, 9 consensus, 3 références, rejets 409.</x:v>
       </x:c>
       <x:c r="H24" s="69" t="str">
-        <x:v>Sources exécutées sans annotations de types et page HTML de test. Frontend compilé et D1 déployé non validés.</x:v>
+        <x:v>Cette suite utilise une page HTML de test. Portable compilé vérifié séparément. Aucun backend D1 déployé validé.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="65" customHeight="1">
@@ -2223,7 +2231,7 @@
         <x:v>Sessions client SessionScope</x:v>
       </x:c>
       <x:c r="C25" s="63" t="str">
-        <x:v>Réussi localement</x:v>
+        <x:v>Réussi localement et en CI</x:v>
       </x:c>
       <x:c r="D25" s="68" t="n">
         <x:v>60</x:v>
@@ -2243,305 +2251,357 @@
     </x:row>
     <x:row r="26" ht="65" customHeight="1">
       <x:c r="A26" s="69" t="str">
-        <x:v>BUILD</x:v>
+        <x:v>RADIO_UI</x:v>
       </x:c>
       <x:c r="B26" s="69" t="str">
-        <x:v>Typage et compilation</x:v>
+        <x:v>Actions radio</x:v>
       </x:c>
       <x:c r="C26" s="69" t="str">
-        <x:v>En attente CI</x:v>
-      </x:c>
-      <x:c r="D26" s="70"/>
-      <x:c r="E26" s="70"/>
+        <x:v>Réussi en CI</x:v>
+      </x:c>
+      <x:c r="D26" s="70" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E26" s="70" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F26" s="72" t="str">
-        <x:v>npm run typecheck ; npm run build:local ; npm run test:portable</x:v>
+        <x:v>node tests/radio-actions.test.mjs</x:v>
       </x:c>
       <x:c r="G26" s="69" t="str">
-        <x:v>Typage, compilation et contrôle du portable compilé restent à valider en CI.</x:v>
+        <x:v>Quatre tests d'actions radio réussis dans le run du commit testé.</x:v>
       </x:c>
       <x:c r="H26" s="69" t="str">
-        <x:v>Le test HTTP depuis les sources ne remplace pas la compilation du frontend.</x:v>
+        <x:v>Actions contrôlées dans la suite automatisée. Aucune écoute humaine validée.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="65" customHeight="1">
       <x:c r="A27" s="63" t="str">
-        <x:v>CI</x:v>
+        <x:v>CONFIG</x:v>
       </x:c>
       <x:c r="B27" s="63" t="str">
-        <x:v>CI du commit livré</x:v>
+        <x:v>Configuration radio</x:v>
       </x:c>
       <x:c r="C27" s="63" t="str">
-        <x:v>En attente CI</x:v>
-      </x:c>
-      <x:c r="D27" s="68"/>
-      <x:c r="E27" s="68"/>
+        <x:v>Réussi en CI</x:v>
+      </x:c>
+      <x:c r="D27" s="68" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E27" s="68" t="n">
+        <x:v>59</x:v>
+      </x:c>
       <x:c r="F27" s="71" t="str">
-        <x:v>GitHub Actions sur la PR 2</x:v>
+        <x:v>npm run test:radio-config</x:v>
       </x:c>
       <x:c r="G27" s="63" t="str">
-        <x:v>En attente sur le commit publié. La CI doit aussi vérifier 4 tests d'actions radio, 59 de configuration et 11 de scène.</x:v>
+        <x:v>59 tests de configuration et de précontrôle radio réussis.</x:v>
       </x:c>
       <x:c r="H27" s="63" t="str">
-        <x:v>Aucun résultat de CI attribué avant exécution sur le commit exact. La scène CPU ne valide pas le GPU.</x:v>
+        <x:v>La configuration validée ne prouve pas la disponibilité d'un relais TURN réel.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="65" customHeight="1">
       <x:c r="A28" s="69" t="str">
-        <x:v>GPU</x:v>
+        <x:v>SCENE_CPU</x:v>
       </x:c>
       <x:c r="B28" s="69" t="str">
-        <x:v>GPU et reflets</x:v>
+        <x:v>Contrôles de scène CPU</x:v>
       </x:c>
       <x:c r="C28" s="69" t="str">
-        <x:v>Non exécuté</x:v>
-      </x:c>
-      <x:c r="D28" s="70"/>
-      <x:c r="E28" s="70"/>
+        <x:v>Réussi en CI</x:v>
+      </x:c>
+      <x:c r="D28" s="70" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E28" s="70" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="F28" s="72" t="str">
-        <x:v>Essai matériel</x:v>
+        <x:v>npm run test:scene</x:v>
       </x:c>
       <x:c r="G28" s="69" t="str">
-        <x:v>Aucun contrôle GPU revendiqué dans cette passe.</x:v>
+        <x:v>11 contrôles CPU supplémentaires réussis, distincts des 234 tests Node.</x:v>
       </x:c>
       <x:c r="H28" s="69" t="str">
-        <x:v>Corps, reflets, anomalies et performances restent à vérifier visuellement.</x:v>
+        <x:v>Ne valide ni pixels GPU, ni qualité des reflets, ni performances graphiques sur appareil.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="65" customHeight="1">
       <x:c r="A29" s="63" t="str">
-        <x:v>MIC</x:v>
+        <x:v>BUILD</x:v>
       </x:c>
       <x:c r="B29" s="63" t="str">
-        <x:v>Microphones réels</x:v>
+        <x:v>Typage et compilation portable</x:v>
       </x:c>
       <x:c r="C29" s="63" t="str">
-        <x:v>Non exécuté</x:v>
+        <x:v>Réussi en CI</x:v>
       </x:c>
       <x:c r="D29" s="68"/>
       <x:c r="E29" s="68"/>
       <x:c r="F29" s="71" t="str">
-        <x:v>Essai matériel</x:v>
+        <x:v>npm run typecheck ; npm run build:local</x:v>
       </x:c>
       <x:c r="G29" s="63" t="str">
-        <x:v>Aucun essai de voix réelle revendiqué.</x:v>
+        <x:v>Étapes TypeScript et build:local réussies sous Node 22.23.4 sur le commit f258c5b6.</x:v>
       </x:c>
       <x:c r="H29" s="63" t="str">
-        <x:v>Intelligibilité, permission, coupure et reprise à tester sur appareils.</x:v>
+        <x:v>Compilation portable. Aucun déploiement du Site ni backend D1 de production validé.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="65" customHeight="1">
       <x:c r="A30" s="69" t="str">
+        <x:v>PORTABLE</x:v>
+      </x:c>
+      <x:c r="B30" s="69" t="str">
+        <x:v>Vérifications du portable compilé</x:v>
+      </x:c>
+      <x:c r="C30" s="69" t="str">
+        <x:v>Réussi en CI</x:v>
+      </x:c>
+      <x:c r="D30" s="70" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E30" s="70" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F30" s="72" t="str">
+        <x:v>npm run test:portable</x:v>
+      </x:c>
+      <x:c r="G30" s="69" t="str">
+        <x:v>11 vérifications réussies avec 2 clients du portable compilé : contexte absent, doublon next, vote ancien rejetés en 409 et départ.</x:v>
+      </x:c>
+      <x:c r="H30" s="69" t="str">
+        <x:v>Protocole du portable compilé vérifié. Pas de partie humaine, de rendu GPU ou de voix réelle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="65" customHeight="1">
+      <x:c r="A31" s="63" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="B31" s="63" t="str">
+        <x:v>CI du commit de code (jobs)</x:v>
+      </x:c>
+      <x:c r="C31" s="63" t="str">
+        <x:v>Réussi en CI</x:v>
+      </x:c>
+      <x:c r="D31" s="68" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E31" s="68" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F31" s="71" t="str">
+        <x:v>https://github.com/darknigthmare/Parallaxe_Protocole9/actions/runs/40884677504</x:v>
+      </x:c>
+      <x:c r="G31" s="63" t="str">
+        <x:v>Run 40884677504 réussi sur f258c5b6bd99e24d6ef9650941fa6a86b162a1f0. 234 tests Node, 11 contrôles CPU et 11 vérifications portable réussis.</x:v>
+      </x:c>
+      <x:c r="H31" s="63" t="str">
+        <x:v>Preuve attachée au commit de code exact. La mise à jour documentaire du suivi est un commit distinct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="65" customHeight="1">
+      <x:c r="A32" s="69" t="str">
+        <x:v>GPU</x:v>
+      </x:c>
+      <x:c r="B32" s="69" t="str">
+        <x:v>GPU et reflets</x:v>
+      </x:c>
+      <x:c r="C32" s="69" t="str">
+        <x:v>Non exécuté</x:v>
+      </x:c>
+      <x:c r="D32" s="70"/>
+      <x:c r="E32" s="70"/>
+      <x:c r="F32" s="72" t="str">
+        <x:v>Essai matériel</x:v>
+      </x:c>
+      <x:c r="G32" s="69" t="str">
+        <x:v>Aucun contrôle GPU revendiqué dans cette passe.</x:v>
+      </x:c>
+      <x:c r="H32" s="69" t="str">
+        <x:v>Corps, reflets, anomalies et performances restent à vérifier visuellement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="65" customHeight="1">
+      <x:c r="A33" s="63" t="str">
+        <x:v>MIC</x:v>
+      </x:c>
+      <x:c r="B33" s="63" t="str">
+        <x:v>Microphones réels</x:v>
+      </x:c>
+      <x:c r="C33" s="63" t="str">
+        <x:v>Non exécuté</x:v>
+      </x:c>
+      <x:c r="D33" s="68"/>
+      <x:c r="E33" s="68"/>
+      <x:c r="F33" s="71" t="str">
+        <x:v>Essai matériel</x:v>
+      </x:c>
+      <x:c r="G33" s="63" t="str">
+        <x:v>Aucun essai de voix réelle revendiqué.</x:v>
+      </x:c>
+      <x:c r="H33" s="63" t="str">
+        <x:v>Intelligibilité, permission, coupure et reprise à tester sur appareils.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="65" customHeight="1">
+      <x:c r="A34" s="69" t="str">
         <x:v>TURN</x:v>
       </x:c>
-      <x:c r="B30" s="69" t="str">
+      <x:c r="B34" s="69" t="str">
         <x:v>TURN entre réseaux</x:v>
       </x:c>
-      <x:c r="C30" s="69" t="str">
+      <x:c r="C34" s="69" t="str">
         <x:v>Non exécuté</x:v>
       </x:c>
-      <x:c r="D30" s="70"/>
-      <x:c r="E30" s="70"/>
-      <x:c r="F30" s="72" t="str">
+      <x:c r="D34" s="70"/>
+      <x:c r="E34" s="70"/>
+      <x:c r="F34" s="72" t="str">
         <x:v>Essai matériel</x:v>
       </x:c>
-      <x:c r="G30" s="69" t="str">
+      <x:c r="G34" s="69" t="str">
         <x:v>Aucune connexion relayée entre réseaux vérifiée.</x:v>
       </x:c>
-      <x:c r="H30" s="69" t="str">
+      <x:c r="H34" s="69" t="str">
         <x:v>Tester avec un relais configuré et deux réseaux distincts.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="22" customHeight="1">
-      <x:c r="A31" s="52"/>
-      <x:c r="B31" s="52"/>
-      <x:c r="C31" s="52"/>
-      <x:c r="D31" s="52"/>
-      <x:c r="E31" s="52"/>
-      <x:c r="F31" s="52"/>
-      <x:c r="G31" s="52"/>
-      <x:c r="H31" s="52"/>
-    </x:row>
-    <x:row r="32" ht="22" customHeight="1">
-      <x:c r="A32" s="52"/>
-      <x:c r="B32" s="52"/>
-      <x:c r="C32" s="52"/>
-      <x:c r="D32" s="52"/>
-      <x:c r="E32" s="52"/>
-      <x:c r="F32" s="52"/>
-      <x:c r="G32" s="52"/>
-      <x:c r="H32" s="52"/>
-    </x:row>
-    <x:row r="33" ht="22" customHeight="1">
-      <x:c r="A33" s="66" t="str">
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="52"/>
+      <x:c r="B35" s="52"/>
+      <x:c r="C35" s="52"/>
+      <x:c r="D35" s="52"/>
+      <x:c r="E35" s="52"/>
+      <x:c r="F35" s="52"/>
+      <x:c r="G35" s="52"/>
+      <x:c r="H35" s="52"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="52"/>
+      <x:c r="B36" s="52"/>
+      <x:c r="C36" s="52"/>
+      <x:c r="D36" s="52"/>
+      <x:c r="E36" s="52"/>
+      <x:c r="F36" s="52"/>
+      <x:c r="G36" s="52"/>
+      <x:c r="H36" s="52"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="66" t="str">
         <x:v>ÉCART DE SOURCES À RÉCONCILIER</x:v>
       </x:c>
-      <x:c r="B33" s="66"/>
-      <x:c r="C33" s="66"/>
-      <x:c r="D33" s="66"/>
-      <x:c r="E33" s="66"/>
-      <x:c r="F33" s="66"/>
-      <x:c r="G33" s="66"/>
-      <x:c r="H33" s="66"/>
-    </x:row>
-    <x:row r="34" ht="30" customHeight="1">
-      <x:c r="A34" s="62" t="str">
+      <x:c r="B37" s="66"/>
+      <x:c r="C37" s="66"/>
+      <x:c r="D37" s="66"/>
+      <x:c r="E37" s="66"/>
+      <x:c r="F37" s="66"/>
+      <x:c r="G37" s="66"/>
+      <x:c r="H37" s="66"/>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="62" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="B34" s="62" t="str">
+      <x:c r="B38" s="62" t="str">
         <x:v>Version</x:v>
       </x:c>
-      <x:c r="C34" s="62" t="str">
+      <x:c r="C38" s="62" t="str">
         <x:v>Lieux annoncés</x:v>
       </x:c>
-      <x:c r="D34" s="62" t="str">
+      <x:c r="D38" s="62" t="str">
         <x:v>Version sauvegardée</x:v>
       </x:c>
-      <x:c r="E34" s="62" t="str">
+      <x:c r="E38" s="62" t="str">
         <x:v>Preuve disponible</x:v>
       </x:c>
-      <x:c r="F34" s="62" t="str">
+      <x:c r="F38" s="62" t="str">
         <x:v>Limite</x:v>
       </x:c>
-      <x:c r="G34" s="62" t="str">
+      <x:c r="G38" s="62" t="str">
         <x:v>Suite</x:v>
       </x:c>
-      <x:c r="H34" s="62" t="str">
+      <x:c r="H38" s="62" t="str">
         <x:v>Référence</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="81" customHeight="1">
-      <x:c r="A35" s="63" t="str">
+    <x:row r="39" ht="81" customHeight="1">
+      <x:c r="A39" s="63" t="str">
         <x:v>GitHub</x:v>
       </x:c>
-      <x:c r="B35" s="63" t="str">
+      <x:c r="B39" s="63" t="str">
         <x:v>0.2.1</x:v>
       </x:c>
-      <x:c r="C35" s="68" t="n">
+      <x:c r="C39" s="68" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D35" s="68"/>
-      <x:c r="E35" s="71" t="str">
+      <x:c r="D39" s="68"/>
+      <x:c r="E39" s="71" t="str">
         <x:v>Code du dépôt examiné à partir de la base indiquée.</x:v>
       </x:c>
-      <x:c r="F35" s="63" t="str">
+      <x:c r="F39" s="63" t="str">
         <x:v>La version GitHub ne prouve pas le contenu du Site 0.4.0.</x:v>
       </x:c>
-      <x:c r="G35" s="63" t="str">
+      <x:c r="G39" s="63" t="str">
         <x:v>Conserver la base des correctifs isolés.</x:v>
       </x:c>
-      <x:c r="H35" s="63" t="str">
+      <x:c r="H39" s="63" t="str">
         <x:v>package.json
 src/game/levels.ts</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="81" customHeight="1">
-      <x:c r="A36" s="73" t="str">
+    <x:row r="40" ht="81" customHeight="1">
+      <x:c r="A40" s="73" t="str">
         <x:v>Site</x:v>
       </x:c>
-      <x:c r="B36" s="73" t="str">
+      <x:c r="B40" s="73" t="str">
         <x:v>0.4.0</x:v>
       </x:c>
-      <x:c r="C36" s="74" t="n">
+      <x:c r="C40" s="74" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D36" s="74" t="n">
+      <x:c r="D40" s="74" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="E36" s="75" t="str">
+      <x:c r="E40" s="75" t="str">
         <x:v>Métadonnées et texte capturé le 28 octobre. Chalet de service affiché.</x:v>
       </x:c>
-      <x:c r="F36" s="73" t="str">
+      <x:c r="F40" s="73" t="str">
         <x:v>Code non récupéré. La version sauvegardée 7 ne prouve pas la version actuellement déployée. Accès réseau bloqué.</x:v>
       </x:c>
-      <x:c r="G36" s="73" t="str">
+      <x:c r="G40" s="73" t="str">
         <x:v>Récupérer le code ou une archive, puis comparer avant remplacement du Site.</x:v>
       </x:c>
-      <x:c r="H36" s="73" t="str">
+      <x:c r="H40" s="73" t="str">
         <x:v>6c8784e0cf5d64f6386f3448434b0bc659d3fc15</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="22" customHeight="1">
-      <x:c r="A37" s="52"/>
-      <x:c r="B37" s="52"/>
-      <x:c r="C37" s="52"/>
-      <x:c r="D37" s="52"/>
-      <x:c r="E37" s="52"/>
-      <x:c r="F37" s="52"/>
-      <x:c r="G37" s="52"/>
-      <x:c r="H37" s="52"/>
-    </x:row>
-    <x:row r="38" ht="22" customHeight="1">
-      <x:c r="A38" s="52"/>
-      <x:c r="B38" s="52"/>
-      <x:c r="C38" s="52"/>
-      <x:c r="D38" s="52"/>
-      <x:c r="E38" s="52"/>
-      <x:c r="F38" s="52"/>
-      <x:c r="G38" s="52"/>
-      <x:c r="H38" s="52"/>
-    </x:row>
-    <x:row r="39" ht="22" customHeight="1">
-      <x:c r="A39" s="76" t="str">
-        <x:v>Livraison</x:v>
-      </x:c>
-      <x:c r="B39" s="77" t="str">
-        <x:v>Pas de fusion ni de déploiement dans cette passe.</x:v>
-      </x:c>
-      <x:c r="C39" s="77"/>
-      <x:c r="D39" s="77"/>
-      <x:c r="E39" s="77"/>
-      <x:c r="F39" s="77"/>
-      <x:c r="G39" s="77"/>
-      <x:c r="H39" s="77"/>
-    </x:row>
-    <x:row r="40" ht="22" customHeight="1">
-      <x:c r="A40" s="76" t="str">
-        <x:v>Classeur source</x:v>
-      </x:c>
-      <x:c r="B40" s="77" t="str">
-        <x:v>docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx</x:v>
-      </x:c>
-      <x:c r="C40" s="77"/>
-      <x:c r="D40" s="77"/>
-      <x:c r="E40" s="77"/>
-      <x:c r="F40" s="77"/>
-      <x:c r="G40" s="77"/>
-      <x:c r="H40" s="77"/>
-    </x:row>
     <x:row r="41" ht="22" customHeight="1">
-      <x:c r="A41" s="76" t="str">
-        <x:v>Empreinte Git</x:v>
-      </x:c>
-      <x:c r="B41" s="77" t="str">
-        <x:v>27846a00639f0611e2ee4b4eaff2e653769a0e16</x:v>
-      </x:c>
-      <x:c r="C41" s="77"/>
-      <x:c r="D41" s="77"/>
-      <x:c r="E41" s="77"/>
-      <x:c r="F41" s="77"/>
-      <x:c r="G41" s="77"/>
-      <x:c r="H41" s="77"/>
+      <x:c r="A41" s="52"/>
+      <x:c r="B41" s="52"/>
+      <x:c r="C41" s="52"/>
+      <x:c r="D41" s="52"/>
+      <x:c r="E41" s="52"/>
+      <x:c r="F41" s="52"/>
+      <x:c r="G41" s="52"/>
+      <x:c r="H41" s="52"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
-      <x:c r="A42" s="76" t="str">
-        <x:v>Suivi détaillé</x:v>
-      </x:c>
-      <x:c r="B42" s="77" t="str">
-        <x:v>docs/suivi-correctifs-20261029.json</x:v>
-      </x:c>
-      <x:c r="C42" s="77"/>
-      <x:c r="D42" s="77"/>
-      <x:c r="E42" s="77"/>
-      <x:c r="F42" s="77"/>
-      <x:c r="G42" s="77"/>
-      <x:c r="H42" s="77"/>
+      <x:c r="A42" s="52"/>
+      <x:c r="B42" s="52"/>
+      <x:c r="C42" s="52"/>
+      <x:c r="D42" s="52"/>
+      <x:c r="E42" s="52"/>
+      <x:c r="F42" s="52"/>
+      <x:c r="G42" s="52"/>
+      <x:c r="H42" s="52"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="76" t="str">
-        <x:v>Preuve manquante</x:v>
+        <x:v>Livraison</x:v>
       </x:c>
       <x:c r="B43" s="77" t="str">
-        <x:v>Les cellules numériques vides correspondent à un résultat non disponible ou à un essai non exécuté, pas à zéro réussite.</x:v>
+        <x:v>Pas de fusion ni de déploiement dans cette passe.</x:v>
       </x:c>
       <x:c r="C43" s="77"/>
       <x:c r="D43" s="77"/>
@@ -2552,10 +2612,10 @@
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="76" t="str">
-        <x:v>Sources</x:v>
+        <x:v>Classeur source</x:v>
       </x:c>
       <x:c r="B44" s="77" t="str">
-        <x:v>docs/SOURCE_RECONCILIATION_2026-10-29.md</x:v>
+        <x:v>docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx</x:v>
       </x:c>
       <x:c r="C44" s="77"/>
       <x:c r="D44" s="77"/>
@@ -2566,10 +2626,10 @@
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="76" t="str">
-        <x:v>QA</x:v>
+        <x:v>Empreinte Git</x:v>
       </x:c>
       <x:c r="B45" s="77" t="str">
-        <x:v>docs/QA.md</x:v>
+        <x:v>27846a00639f0611e2ee4b4eaff2e653769a0e16</x:v>
       </x:c>
       <x:c r="C45" s="77"/>
       <x:c r="D45" s="77"/>
@@ -2578,12 +2638,68 @@
       <x:c r="G45" s="77"/>
       <x:c r="H45" s="77"/>
     </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="76" t="str">
+        <x:v>Suivi détaillé</x:v>
+      </x:c>
+      <x:c r="B46" s="77" t="str">
+        <x:v>docs/suivi-correctifs-20261029.json</x:v>
+      </x:c>
+      <x:c r="C46" s="77"/>
+      <x:c r="D46" s="77"/>
+      <x:c r="E46" s="77"/>
+      <x:c r="F46" s="77"/>
+      <x:c r="G46" s="77"/>
+      <x:c r="H46" s="77"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="76" t="str">
+        <x:v>Preuve manquante</x:v>
+      </x:c>
+      <x:c r="B47" s="77" t="str">
+        <x:v>Les cellules numériques vides correspondent à un résultat non disponible ou à un essai non exécuté, pas à zéro réussite.</x:v>
+      </x:c>
+      <x:c r="C47" s="77"/>
+      <x:c r="D47" s="77"/>
+      <x:c r="E47" s="77"/>
+      <x:c r="F47" s="77"/>
+      <x:c r="G47" s="77"/>
+      <x:c r="H47" s="77"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="76" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="B48" s="77" t="str">
+        <x:v>docs/SOURCE_RECONCILIATION_2026-10-29.md</x:v>
+      </x:c>
+      <x:c r="C48" s="77"/>
+      <x:c r="D48" s="77"/>
+      <x:c r="E48" s="77"/>
+      <x:c r="F48" s="77"/>
+      <x:c r="G48" s="77"/>
+      <x:c r="H48" s="77"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="76" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="B49" s="77" t="str">
+        <x:v>docs/QA.md</x:v>
+      </x:c>
+      <x:c r="C49" s="77"/>
+      <x:c r="D49" s="77"/>
+      <x:c r="E49" s="77"/>
+      <x:c r="F49" s="77"/>
+      <x:c r="G49" s="77"/>
+      <x:c r="H49" s="77"/>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C9:C16">
     <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Bloqué"/>
     <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="en cours"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="C21:C30">
+  <x:conditionalFormatting sqref="C21:C34">
     <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="En cours"/>
     <x:cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="En attente"/>
     <x:cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Non validé"/>
@@ -2591,7 +2707,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19bd297353c241ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc45d4d8e07124fc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: track control and reflection fixes without overstating queued CI
Add dated gameplay and package tracking, preserve the three existing workbook sheets, and record V8 reproductions separately from the pending Node, build and extracted ZIP gates.
Reference input-systems and clarify revision-specific CI packages and the still unavailable Site 0.4.0 source.
</commit_message>
<xml_diff>
--- a/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
+++ b/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
@@ -5,6 +5,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R0b19b9158c464378"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="2" r:id="Rf274adb891e642e6"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctifs 29-10" sheetId="3" r:id="R1daed0cc66c3480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jouabilité 29-10" sheetId="4" r:id="RParallaxeJouabilite20261029"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2710,4 +2711,476 @@
     <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc45d4d8e07124fc8"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF3E756F"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="18"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" customWidth="1"/>
+    <x:col min="2" max="2" width="31" customWidth="1"/>
+    <x:col min="3" max="3" width="27" customWidth="1"/>
+    <x:col min="4" max="4" width="48" customWidth="1"/>
+    <x:col min="5" max="5" width="56" customWidth="1"/>
+    <x:col min="6" max="6" width="49" customWidth="1"/>
+    <x:col min="7" max="7" width="45" customWidth="1"/>
+    <x:col min="8" max="8" width="48" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="54" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PARALLAXE — JOUABILITÉ ET PAQUET PC</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="56" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Reprise du 29 octobre 2026 · Base GitHub 0.2.1 · PR #2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="52" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Révision du lot</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="52" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">b70350c59e97487d0c7224d6c57c17eabb0f8e1b</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="52" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="52" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="52" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CI</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="52" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://github.com/darknigthmare/Parallaxe_Protocole9/actions/runs/40901665020</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="40" customHeight="1">
+      <x:c r="A4" s="63" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Résultats</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="63" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">5 points implémentés · CI GitHub en attente · simulations V8 réussies · récupération 0.4.0 et essais sur appareil encore ouverts</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="32" customHeight="1">
+      <x:c r="A5" s="58" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Les trois feuilles précédentes conservent leur contenu et leurs preuves historiques. La validation sur appareil reste distincte.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="32" customHeight="1">
+      <x:c r="A6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Correction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Statut</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Critère de validation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Preuve</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Limite</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Suite</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" s="62" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sources du lot</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="112" customHeight="1">
+      <x:c r="A7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Interruption des gestes de déplacement et de regard</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Les interruptions et les anciens événements ne réactivent ni mouvement ni regard ; un nouveau geste et deux doigts indépendants restent fonctionnels.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">npm run test:movement
+npm run test:session-client</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Callbacks réels avec frontières navigateur simulées.
+React et périphérique tactile réel non testés.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">app/game.tsx
+tests/movement-input.test.mjs
+tests/session-scope.test.mjs</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="112" customHeight="1">
+      <x:c r="A8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Retour de l'épaule après le talkie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Repos, marche, mannequin et état normal après radio retrouvent la pose d'un inspecteur neuf ; le geste indépendant fonctionne toujours.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">npm run test:scene</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Transformations CPU vérifiées ; rendu des avatars et des reflets sur GPU restant à examiner.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">src/game/avatar.ts
+tests/scene.geometry.test.mjs</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="112" customHeight="1">
+      <x:c r="A9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Durée du reflet retardé à haute fréquence</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Une seconde de décalage est conservée à 20, 60, 120, 240, 360 Hz et en cadence variable, à la résolution d'échantillonnage près.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">npm run test:scene</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Cadences simulées dans la scène CPU ; aucune mesure de FPS sur écran ou GPU.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">src/game/scene.ts
+tests/scene.geometry.test.mjs</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="112" customHeight="1">
+      <x:c r="A10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Paquet PC lancé depuis son ZIP extrait</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Le ZIP testé démarre sans node_modules ; les décisions coopératives et les rejets de requêtes périmées réussissent.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">npm run package:release
+python3 tests/package-archive.test.py</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Serveur et clients HTTP sous Linux ; rendu du navigateur et lanceur Windows non exécutés.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">scripts/package-release.mjs
+tests/package-archive.test.py
+tests/portable.test.mjs
+.github/workflows/ci.yml</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="112" customHeight="1">
+      <x:c r="A11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Révision commune aux tests et archives</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">La révision des deux checkouts, COMMIT.txt et le manifeste correspondent ; les artefacts ne sont publiés qu'après validation.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">GitHub Actions: source-snapshot
+GitHub Actions: game</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Les archives historiques suivies dans public/downloads conservent leur contenu antérieur.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">.github/workflows/ci.yml
+scripts/package-release.mjs</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="112" customHeight="1">
+      <x:c r="A12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Réconcilier le Site 0.4.0 avec GitHub</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bloqué</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Récupérer les fichiers sources via la reprise Sites, comparer les deux versions et reporter les correctifs sur la source finale.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Relevé des sources et limites</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exécuteur indisponible pour reprendre le dépôt Sites.
+Aucun code 0.4.0 récupéré ; aucun déploiement effectué.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Récupérer et comparer le dépôt Sites</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/SOURCE_RECONCILIATION_2026-10-29.md</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="112" customHeight="1">
+      <x:c r="A13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JOU07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Validation sur les appareils cibles</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">À valider sur appareil</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Jouer sur GPU et écran tactile, vérifier les inspecteurs/reflets puis microphones et relais TURN.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Relevé des sources et limites</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Essais matériels non exécutés dans ce lot.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Essais sur les appareils cibles</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" s="64" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/QA.md</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="63" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Méthode</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="63" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Essais automatiques sur le commit indiqué. Les corps des callbacks, la scène CPU et le paquet extrait sont vérifiés séparément.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="63" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sur cible</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="63" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rendu GPU, écran tactile physique, micros et relais TURN : essais non exécutés dans ce lot.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:autoFilter ref="A6:H13"/>
+  <x:mergeCells count="8">
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="B3:D3"/>
+    <x:mergeCell ref="F3:H3"/>
+    <x:mergeCell ref="B4:H4"/>
+    <x:mergeCell ref="A5:H5"/>
+    <x:mergeCell ref="B15:H15"/>
+    <x:mergeCell ref="B16:H16"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <x:pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Livrer les archives 0.4.1 testées et consigner la publication privée
</commit_message>
<xml_diff>
--- a/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
+++ b/docs/PARALLAXE_Suivi_Reprise_2026-10-28.xlsx
@@ -2714,473 +2714,440 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetPr>
-    <x:tabColor rgb="FF3E756F"/>
-  </x:sheetPr>
-  <x:sheetFormatPr defaultRowHeight="18"/>
-  <x:cols>
-    <x:col min="1" max="1" width="14" customWidth="1"/>
-    <x:col min="2" max="2" width="31" customWidth="1"/>
-    <x:col min="3" max="3" width="27" customWidth="1"/>
-    <x:col min="4" max="4" width="48" customWidth="1"/>
-    <x:col min="5" max="5" width="56" customWidth="1"/>
-    <x:col min="6" max="6" width="49" customWidth="1"/>
-    <x:col min="7" max="7" width="45" customWidth="1"/>
-    <x:col min="8" max="8" width="48" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="54" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PARALLAXE — JOUABILITÉ ET PAQUET PC</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Reprise du 29 octobre 2026 · Base GitHub 0.2.1 · PR #2</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Révision du lot</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">b70350c59e97487d0c7224d6c57c17eabb0f8e1b</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CI</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://github.com/darknigthmare/Parallaxe_Protocole9/actions/runs/40901665020</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="40" customHeight="1">
-      <x:c r="A4" s="63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Résultats</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5 points implémentés · CI GitHub en attente · simulations V8 réussies · récupération 0.4.0 et essais sur appareil encore ouverts</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="32" customHeight="1">
-      <x:c r="A5" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Les trois feuilles précédentes conservent leur contenu et leurs preuves historiques. La validation sur appareil reste distincte.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ID</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Correction</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Statut</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Critère de validation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Preuve</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Limite</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Suite</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H6" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sources du lot</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="112" customHeight="1">
-      <x:c r="A7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Interruption des gestes de déplacement et de regard</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Les interruptions et les anciens événements ne réactivent ni mouvement ni regard ; un nouveau geste et deux doigts indépendants restent fonctionnels.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">npm run test:movement
-npm run test:session-client</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Callbacks réels avec frontières navigateur simulées.
-React et périphérique tactile réel non testés.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H7" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">app/game.tsx
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF3E756F"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="56" customWidth="1"/>
+    <col min="6" max="6" width="49" customWidth="1"/>
+    <col min="7" max="7" width="45" customWidth="1"/>
+    <col min="8" max="8" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARALLAXE — JOUABILITÉ ET PAQUET PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="56" t="str">
+        <v>Reprise du 29 octobre 2026 · Version 0.4.1 consolidée dans la PR #2</v>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Révision du lot</t>
+        </is>
+      </c>
+      <c r="B3" s="52" t="str">
+        <v>fa9cf6306705c750106467d0d6caddf96767b0e7</v>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CI</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="str">
+        <v>https://github.com/darknigthmare/Parallaxe_Protocole9/actions/runs/40907389674</v>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Résultats</t>
+        </is>
+      </c>
+      <c r="B4" s="63" t="str">
+        <v>334 contrôles locaux réussis : 281 tests Node, 31 de scène, 9 du chalet et 13 d’inspection. Builds et ZIP validés. Site privé publié. CI en attente.</v>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="58" t="str">
+        <v>Sources Site 0.4.0 récupérées et intégrées. La version 0.4.1 est publiée en accès privé. Les trois feuilles précédentes conservent leurs preuves historiques.</v>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correction</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statut</t>
+        </is>
+      </c>
+      <c r="D6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critère de validation</t>
+        </is>
+      </c>
+      <c r="E6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preuve</t>
+        </is>
+      </c>
+      <c r="F6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limite</t>
+        </is>
+      </c>
+      <c r="G6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suite</t>
+        </is>
+      </c>
+      <c r="H6" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sources du lot</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="64" t="str">
+        <v>JOU01</v>
+      </c>
+      <c r="B7" s="64" t="str">
+        <v>Gestes interrompus et reprise de session</v>
+      </c>
+      <c r="C7" s="64" t="str">
+        <v>Vérifié localement</v>
+      </c>
+      <c r="D7" s="64" t="str">
+        <v>Une pause, une modale, un verdict ou une perte de focus annule les gestes. Les pointeurs restent indépendants et les anciennes réponses de session sont ignorées.</v>
+      </c>
+      <c r="E7" s="64" t="str">
+        <v>test:movement : 28/28
+test:session-client : 64/64
+npm test : 165/165 au total</v>
+      </c>
+      <c r="F7" s="64" t="str">
+        <v>Callbacks réels, navigateur simulé.
+React et tactile physique non exécutés.</v>
+      </c>
+      <c r="G7" s="64" t="str">
+        <v>Confirmer la CI puis essayer les commandes sur appareil.</v>
+      </c>
+      <c r="H7" s="64" t="str">
+        <v>app/game.tsx
 tests/movement-input.test.mjs
-tests/session-scope.test.mjs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="112" customHeight="1">
-      <x:c r="A8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Retour de l'épaule après le talkie</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Repos, marche, mannequin et état normal après radio retrouvent la pose d'un inspecteur neuf ; le geste indépendant fonctionne toujours.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">npm run test:scene</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Transformations CPU vérifiées ; rendu des avatars et des reflets sur GPU restant à examiner.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H8" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/game/avatar.ts
-tests/scene.geometry.test.mjs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="112" customHeight="1">
-      <x:c r="A9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Durée du reflet retardé à haute fréquence</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Une seconde de décalage est conservée à 20, 60, 120, 240, 360 Hz et en cadence variable, à la résolution d'échantillonnage près.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">npm run test:scene</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cadences simulées dans la scène CPU ; aucune mesure de FPS sur écran ou GPU.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H9" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/game/scene.ts
-tests/scene.geometry.test.mjs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="112" customHeight="1">
-      <x:c r="A10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU04</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Paquet PC lancé depuis son ZIP extrait</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Le ZIP testé démarre sans node_modules ; les décisions coopératives et les rejets de requêtes périmées réussissent.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">npm run package:release
-python3 tests/package-archive.test.py</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Serveur et clients HTTP sous Linux ; rendu du navigateur et lanceur Windows non exécutés.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H10" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">scripts/package-release.mjs
+tests/session-scope.test.mjs</v>
+      </c>
+    </row>
+    <row r="8" ht="112" customHeight="1">
+      <c r="A8" s="64" t="str">
+        <v>JOU02</v>
+      </c>
+      <c r="B8" s="64" t="str">
+        <v>Retour de pose des inspecteurs</v>
+      </c>
+      <c r="C8" s="64" t="str">
+        <v>Vérifié localement</v>
+      </c>
+      <c r="D8" s="64" t="str">
+        <v>Repos, marche, mannequin et état normal après radio retrouvent la pose d’un inspecteur neuf. Le geste indépendant fonctionne toujours.</v>
+      </c>
+      <c r="E8" s="64" t="str">
+        <v>test:scene : 31/31
+Dont cinq régressions de retour de pose.</v>
+      </c>
+      <c r="F8" s="64" t="str">
+        <v>La source 0.4.0 réinitialisait déjà l’axe Y. Les transformations CPU sont vérifiées. Le rendu GPU reste à examiner.</v>
+      </c>
+      <c r="G8" s="64" t="str">
+        <v>Vérifier visuellement les corps et reflets sur appareil.</v>
+      </c>
+      <c r="H8" s="64" t="str">
+        <v>src/game/avatar.ts
+tests/scene.geometry.test.mjs</v>
+      </c>
+    </row>
+    <row r="9" ht="112" customHeight="1">
+      <c r="A9" s="64" t="str">
+        <v>JOU03</v>
+      </c>
+      <c r="B9" s="64" t="str">
+        <v>Retard du reflet à haute fréquence</v>
+      </c>
+      <c r="C9" s="64" t="str">
+        <v>Vérifié localement</v>
+      </c>
+      <c r="D9" s="64" t="str">
+        <v>Une seconde de décalage est conservée à 20, 60, 120, 240, 360 Hz et en cadence variable, à la résolution d’échantillonnage près.</v>
+      </c>
+      <c r="E9" s="64" t="str">
+        <v>test:scene : 31/31
+Un contrôle couvre six cadences.</v>
+      </c>
+      <c r="F9" s="64" t="str">
+        <v>Cadences simulées dans la scène CPU. Aucune mesure de FPS sur écran ou GPU.</v>
+      </c>
+      <c r="G9" s="64" t="str">
+        <v>Observer le reflet sur plusieurs appareils et qualités.</v>
+      </c>
+      <c r="H9" s="64" t="str">
+        <v>src/game/scene.ts
+tests/scene.geometry.test.mjs</v>
+      </c>
+    </row>
+    <row r="10" ht="112" customHeight="1">
+      <c r="A10" s="64" t="str">
+        <v>JOU04</v>
+      </c>
+      <c r="B10" s="64" t="str">
+        <v>Paquet PC depuis son ZIP extrait</v>
+      </c>
+      <c r="C10" s="64" t="str">
+        <v>Vérifié localement</v>
+      </c>
+      <c r="D10" s="64" t="str">
+        <v>Le ZIP démarre sans node_modules. Deux clients puis quatre inspecteurs dans le chalet valident le protocole et les rejets de décisions périmées.</v>
+      </c>
+      <c r="E10" s="64" t="str">
+        <v>build et build:local réussis
+ZIP 0.4.1 : 17 vérifications réussies
+12 requêtes de chemins protégés
+Chalet : 4 clients, 9 diagnostics, victoire</v>
+      </c>
+      <c r="F10" s="64" t="str">
+        <v>Serveur HTTP Linux lancé depuis une extraction neuve. Lanceur Windows, rendu GPU et appareils physiques non exécutés.</v>
+      </c>
+      <c r="G10" s="64" t="str">
+        <v>Confirmer la CI puis essayer le paquet sur Windows et sur GPU.</v>
+      </c>
+      <c r="H10" s="64" t="str">
+        <v>scripts/package-release.mjs
 tests/package-archive.test.py
 tests/portable.test.mjs
-.github/workflows/ci.yml</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="112" customHeight="1">
-      <x:c r="A11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU05</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Révision commune aux tests et archives</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implémenté · CI en attente</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">La révision des deux checkouts, COMMIT.txt et le manifeste correspondent ; les artefacts ne sont publiés qu'après validation.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GitHub Actions: source-snapshot
-GitHub Actions: game</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Les archives historiques suivies dans public/downloads conservent leur contenu antérieur.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmer la CI puis les essais sur cible</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H11" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">.github/workflows/ci.yml
-scripts/package-release.mjs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="112" customHeight="1">
-      <x:c r="A12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU06</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Réconcilier le Site 0.4.0 avec GitHub</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bloqué</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Récupérer les fichiers sources via la reprise Sites, comparer les deux versions et reporter les correctifs sur la source finale.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Relevé des sources et limites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Exécuteur indisponible pour reprendre le dépôt Sites.
-Aucun code 0.4.0 récupéré ; aucun déploiement effectué.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Récupérer et comparer le dépôt Sites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H12" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">docs/SOURCE_RECONCILIATION_2026-10-29.md</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="112" customHeight="1">
-      <x:c r="A13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JOU07</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Validation sur les appareils cibles</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">À valider sur appareil</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Jouer sur GPU et écran tactile, vérifier les inspecteurs/reflets puis microphones et relais TURN.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Relevé des sources et limites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Essais matériels non exécutés dans ce lot.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Essais sur les appareils cibles</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H13" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">docs/QA.md</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="36" customHeight="1">
-      <x:c r="A15" s="63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Méthode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Essais automatiques sur le commit indiqué. Les corps des callbacks, la scène CPU et le paquet extrait sont vérifiés séparément.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="36" customHeight="1">
-      <x:c r="A16" s="63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sur cible</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rendu GPU, écran tactile physique, micros et relais TURN : essais non exécutés dans ce lot.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:autoFilter ref="A6:H13"/>
-  <x:mergeCells count="8">
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="B3:D3"/>
-    <x:mergeCell ref="F3:H3"/>
-    <x:mergeCell ref="B4:H4"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="B15:H15"/>
-    <x:mergeCell ref="B16:H16"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <x:pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>
-</x:worksheet>
+.github/workflows/ci.yml</v>
+      </c>
+    </row>
+    <row r="11" ht="112" customHeight="1">
+      <c r="A11" s="64" t="str">
+        <v>JOU05</v>
+      </c>
+      <c r="B11" s="64" t="str">
+        <v>Révision des tests et des archives</v>
+      </c>
+      <c r="C11" s="64" t="str">
+        <v>Archives vérifiées localement</v>
+      </c>
+      <c r="D11" s="64" t="str">
+        <v>COMMIT.txt et manifeste : révision indiquée.
+Checkout propre. CRC, SHA-256, build complet et sources embarquées vérifiés.</v>
+      </c>
+      <c r="E11" s="64" t="str">
+        <v>SHA-256 PC :
+7b19158d79e326e4bf3b753679221eb2
+7f67dfb1a7ec16b3449ebf366dca21f6
+SHA-256 sources :
+3742644e36e63f47105bb347802fa3f2
+49efbd38d1f4a77839b349bc3e59cb42</v>
+      </c>
+      <c r="F11" s="64" t="str">
+        <v>Checkout propre (dirty: false).
+CI distante : jobs en attente.</v>
+      </c>
+      <c r="G11" s="64" t="str">
+        <v>Confirmer GitHub Actions pour la révision exacte.</v>
+      </c>
+      <c r="H11" s="64" t="str">
+        <v>COMMIT.txt
+SHA256SUMS.txt
+release-manifest.json
+.github/workflows/ci.yml</v>
+      </c>
+    </row>
+    <row r="12" ht="112" customHeight="1">
+      <c r="A12" s="64" t="str">
+        <v>JOU06</v>
+      </c>
+      <c r="B12" s="64" t="str">
+        <v>Sources réconciliées et Site publié</v>
+      </c>
+      <c r="C12" s="64" t="str">
+        <v>Publié en accès privé</v>
+      </c>
+      <c r="D12" s="64" t="str">
+        <v>Le contenu 0.4.0 récupéré et les correctifs de la PR coexistent dans la version 0.4.1 publiée. Les quatre lieux, 96 anomalies et l’accès privé sont conservés.</v>
+      </c>
+      <c r="E12" s="64" t="str">
+        <v>Publication réussie le 29/10/2026 à 17:07 (Paris).
+Source publiée :
+064a2157b64787228966ea108b683f735f2e3dc6</v>
+      </c>
+      <c r="F12" s="64" t="str">
+        <v>Publication confirmée par Sites. Aucun parcours navigateur, rendu GPU ou microphone physique n’est validé par ce déploiement.</v>
+      </c>
+      <c r="G12" s="64" t="str">
+        <v>Confirmer la CI puis effectuer la recette navigateur et sur appareils.</v>
+      </c>
+      <c r="H12" s="64" t="str">
+        <v>https://parallaxe-protocole-neuf.darknigthmare.chatgpt.site
+Déploiement :
+appgdep_6ae36f3e3f848191b1ec1afb032c56e4
+docs/SOURCE_RECONCILIATION_2026-10-29.md</v>
+      </c>
+    </row>
+    <row r="13" ht="112" customHeight="1">
+      <c r="A13" s="64" t="str">
+        <v>JOU07</v>
+      </c>
+      <c r="B13" s="64" t="str">
+        <v>Validation sur les appareils cibles</v>
+      </c>
+      <c r="C13" s="64" t="str">
+        <v>Non exécuté</v>
+      </c>
+      <c r="D13" s="64" t="str">
+        <v>Jouer sur GPU et écran tactile, examiner les inspecteurs et reflets, puis vérifier les microphones et le relais TURN.</v>
+      </c>
+      <c r="E13" s="64" t="str">
+        <v>Aucun essai matériel effectué dans cette passe.</v>
+      </c>
+      <c r="F13" s="64" t="str">
+        <v>CPU et simulations audio ne valident ni les pixels, ni les performances, ni la qualité vocale entre réseaux.</v>
+      </c>
+      <c r="G13" s="64" t="str">
+        <v>Effectuer la recette sur les appareils cibles.</v>
+      </c>
+      <c r="H13" s="64" t="str">
+        <v>docs/QA.md</v>
+      </c>
+    </row>
+    <row r="14" ht="112" customHeight="1">
+      <c r="A14" s="64" t="str">
+        <v>JOU08</v>
+      </c>
+      <c r="B14" s="64" t="str">
+        <v>Calibration radio et annulation</v>
+      </c>
+      <c r="C14" s="64" t="str">
+        <v>Vérifié localement</v>
+      </c>
+      <c r="D14" s="64" t="str">
+        <v>Les douze profils gardent leur preuve de calibration. Arrêter le test, changer de perception ou quitter invalide les préparations et résultats périmés.</v>
+      </c>
+      <c r="E14" s="64" t="str">
+        <v>test:radio : 42/42
+test:radio-ui : 15/15
+test:radio-config : 59/59</v>
+      </c>
+      <c r="F14" s="64" t="str">
+        <v>API audio simulées et signaux PCM synthétiques. Microphone physique, écoute et TURN non exécutés.</v>
+      </c>
+      <c r="G14" s="64" t="str">
+        <v>Vérifier l’écoute réelle et la transmission entre appareils.</v>
+      </c>
+      <c r="H14" s="64" t="str">
+        <v>src/game/radio.ts
+src/game/radio-evidence.ts
+app/game.tsx
+tests/radio.test.mjs</v>
+      </c>
+    </row>
+    <row r="15" ht="112" customHeight="1">
+      <c r="A15" s="64" t="str">
+        <v>JOU09</v>
+      </c>
+      <c r="B15" s="64" t="str">
+        <v>Chalet et catalogue conservés</v>
+      </c>
+      <c r="C15" s="64" t="str">
+        <v>Vérifié localement</v>
+      </c>
+      <c r="D15" s="64" t="str">
+        <v>Le chalet reste un lieu optionnel. La campagne conserve trois secteurs. Les 96 anomalies ont une perception témoin et une référence normale.</v>
+      </c>
+      <c r="E15" s="64" t="str">
+        <v>Règles : 19/19
+Chalet : 9/9
+Inspection : 13/13
+Scène : 31/31</v>
+      </c>
+      <c r="F15" s="64" t="str">
+        <v>Géométries, collisions et lectures privées vérifiées sur CPU. Apparence et confort sur GPU non exécutés.</v>
+      </c>
+      <c r="G15" s="64" t="str">
+        <v>Effectuer la recette visuelle du chalet et la coopération sur appareils.</v>
+      </c>
+      <c r="H15" s="64" t="str">
+        <v>src/game/cabin.ts
+src/game/catalog.ts
+src/game/levels.ts
+tests/cabin.geometry.test.mjs
+tests/inspection.test.mjs</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16"/>
+      <c r="B16"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="63" t="str">
+        <v>Méthode</v>
+      </c>
+      <c r="B17" s="63" t="str">
+        <v>Node.js 24.22.1 local. TypeScript, 334 contrôles et les deux builds réussis. Le paquet extrait ajoute 17 vérifications et 12 requêtes de chemins. CI Node 22 en attente.</v>
+      </c>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="63" t="str">
+        <v>Sur cible</v>
+      </c>
+      <c r="B18" s="63" t="str">
+        <v>Rendu GPU, tactile physique, microphones, écoute réelle et relais TURN : essais non exécutés dans ce lot.</v>
+      </c>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:H15"/>
+  <mergeCells>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
 </file>
</xml_diff>